<commit_message>
Rebuild Assessment 3 regressions with new variables.
Assessment 2 used rank, value, age, titles, host, rest, confederation
and knockout. These models use four new predictors each, with two shared
(World Cup appearances and calendar day).

Co-authored-by: Bhupraj Tamang <BhuprajTmg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/cleaned/fifa_data_cleaned.xlsx
+++ b/data/cleaned/fifa_data_cleaned.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="matches" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="teams" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="players" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="team_roster" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -47541,4 +47542,1702 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>team</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>roster_size</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>n_fw</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>n_mf</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>n_df</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>n_gk</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>youth_share</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>veteran_share</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>age_spread</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>fwd_share</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Algeria</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>22</v>
+      </c>
+      <c r="C2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E2" t="n">
+        <v>7</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.04545454545454546</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.09090909090909091</v>
+      </c>
+      <c r="I2" t="n">
+        <v>3.781934730138835</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.3181818181818182</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>23</v>
+      </c>
+      <c r="C3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.08695652173913043</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.1739130434782609</v>
+      </c>
+      <c r="I3" t="n">
+        <v>4.330697485563088</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.3043478260869565</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>23</v>
+      </c>
+      <c r="C4" t="n">
+        <v>8</v>
+      </c>
+      <c r="D4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.3043478260869565</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.2173913043478261</v>
+      </c>
+      <c r="I4" t="n">
+        <v>5.079603482704332</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.3478260869565217</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" t="n">
+        <v>9</v>
+      </c>
+      <c r="E5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I5" t="n">
+        <v>3.937338133682116</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>23</v>
+      </c>
+      <c r="C6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E6" t="n">
+        <v>7</v>
+      </c>
+      <c r="F6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.1304347826086956</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.3043478260869565</v>
+      </c>
+      <c r="I6" t="n">
+        <v>4.960316832925488</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.2608695652173913</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Bosnia and Herzegovina</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>23</v>
+      </c>
+      <c r="C7" t="n">
+        <v>7</v>
+      </c>
+      <c r="D7" t="n">
+        <v>8</v>
+      </c>
+      <c r="E7" t="n">
+        <v>7</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.2173913043478261</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.08695652173913043</v>
+      </c>
+      <c r="I7" t="n">
+        <v>4.839723638926688</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.3043478260869565</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>19</v>
+      </c>
+      <c r="C8" t="n">
+        <v>9</v>
+      </c>
+      <c r="D8" t="n">
+        <v>6</v>
+      </c>
+      <c r="E8" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.1052631578947368</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.3157894736842105</v>
+      </c>
+      <c r="I8" t="n">
+        <v>4.681055511501053</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.4736842105263158</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>23</v>
+      </c>
+      <c r="C9" t="n">
+        <v>7</v>
+      </c>
+      <c r="D9" t="n">
+        <v>7</v>
+      </c>
+      <c r="E9" t="n">
+        <v>8</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.1304347826086956</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.08695652173913043</v>
+      </c>
+      <c r="I9" t="n">
+        <v>3.396114962415829</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.3043478260869565</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Cape Verde</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>20</v>
+      </c>
+      <c r="C10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" t="n">
+        <v>12</v>
+      </c>
+      <c r="E10" t="n">
+        <v>3</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I10" t="n">
+        <v>4.908639000996637</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>19</v>
+      </c>
+      <c r="C11" t="n">
+        <v>5</v>
+      </c>
+      <c r="D11" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" t="n">
+        <v>8</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.05263157894736842</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.3157894736842105</v>
+      </c>
+      <c r="I11" t="n">
+        <v>3.989020017717934</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.2631578947368421</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>19</v>
+      </c>
+      <c r="C12" t="n">
+        <v>6</v>
+      </c>
+      <c r="D12" t="n">
+        <v>7</v>
+      </c>
+      <c r="E12" t="n">
+        <v>5</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.1052631578947368</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.2631578947368421</v>
+      </c>
+      <c r="I12" t="n">
+        <v>5.556725023109938</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.3157894736842105</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Curacao</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>22</v>
+      </c>
+      <c r="C13" t="n">
+        <v>8</v>
+      </c>
+      <c r="D13" t="n">
+        <v>5</v>
+      </c>
+      <c r="E13" t="n">
+        <v>8</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.04545454545454546</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.2727272727272727</v>
+      </c>
+      <c r="I13" t="n">
+        <v>4.093073020756745</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.3636363636363636</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Czechia</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>21</v>
+      </c>
+      <c r="C14" t="n">
+        <v>6</v>
+      </c>
+      <c r="D14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.1904761904761905</v>
+      </c>
+      <c r="I14" t="n">
+        <v>3.767024846012592</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.2857142857142857</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>DR Congo</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>20</v>
+      </c>
+      <c r="C15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D15" t="n">
+        <v>7</v>
+      </c>
+      <c r="E15" t="n">
+        <v>7</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I15" t="n">
+        <v>3.330876287421263</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>22</v>
+      </c>
+      <c r="C16" t="n">
+        <v>6</v>
+      </c>
+      <c r="D16" t="n">
+        <v>7</v>
+      </c>
+      <c r="E16" t="n">
+        <v>8</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.2272727272727273</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.09090909090909091</v>
+      </c>
+      <c r="I16" t="n">
+        <v>4.576667722905766</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.2727272727272727</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>18</v>
+      </c>
+      <c r="C17" t="n">
+        <v>7</v>
+      </c>
+      <c r="D17" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" t="n">
+        <v>6</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.05555555555555555</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="I17" t="n">
+        <v>3.887721580176148</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.3888888888888889</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>24</v>
+      </c>
+      <c r="C18" t="n">
+        <v>7</v>
+      </c>
+      <c r="D18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E18" t="n">
+        <v>9</v>
+      </c>
+      <c r="F18" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.08333333333333333</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.2083333333333333</v>
+      </c>
+      <c r="I18" t="n">
+        <v>3.915548714947936</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.2916666666666667</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>22</v>
+      </c>
+      <c r="C19" t="n">
+        <v>7</v>
+      </c>
+      <c r="D19" t="n">
+        <v>6</v>
+      </c>
+      <c r="E19" t="n">
+        <v>8</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.1363636363636364</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.04545454545454546</v>
+      </c>
+      <c r="I19" t="n">
+        <v>3.139263983002761</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.3181818181818182</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>23</v>
+      </c>
+      <c r="C20" t="n">
+        <v>4</v>
+      </c>
+      <c r="D20" t="n">
+        <v>10</v>
+      </c>
+      <c r="E20" t="n">
+        <v>8</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.08695652173913043</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.1304347826086956</v>
+      </c>
+      <c r="I20" t="n">
+        <v>4.470810026437058</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.1739130434782609</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>22</v>
+      </c>
+      <c r="C21" t="n">
+        <v>7</v>
+      </c>
+      <c r="D21" t="n">
+        <v>5</v>
+      </c>
+      <c r="E21" t="n">
+        <v>8</v>
+      </c>
+      <c r="F21" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.2727272727272727</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.1363636363636364</v>
+      </c>
+      <c r="I21" t="n">
+        <v>4.040112723985659</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.3181818181818182</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Haiti</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>17</v>
+      </c>
+      <c r="C22" t="n">
+        <v>7</v>
+      </c>
+      <c r="D22" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" t="n">
+        <v>6</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="I22" t="n">
+        <v>4.108814055317723</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.4117647058823529</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Iran</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>18</v>
+      </c>
+      <c r="C23" t="n">
+        <v>5</v>
+      </c>
+      <c r="D23" t="n">
+        <v>6</v>
+      </c>
+      <c r="E23" t="n">
+        <v>6</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.3888888888888889</v>
+      </c>
+      <c r="I23" t="n">
+        <v>3.772968873135194</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.2777777777777778</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Iraq</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>21</v>
+      </c>
+      <c r="C24" t="n">
+        <v>7</v>
+      </c>
+      <c r="D24" t="n">
+        <v>6</v>
+      </c>
+      <c r="E24" t="n">
+        <v>7</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.1904761904761905</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.1428571428571428</v>
+      </c>
+      <c r="I24" t="n">
+        <v>4.011293580688926</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Ivory Coast</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>22</v>
+      </c>
+      <c r="C25" t="n">
+        <v>9</v>
+      </c>
+      <c r="D25" t="n">
+        <v>5</v>
+      </c>
+      <c r="E25" t="n">
+        <v>7</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.2727272727272727</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0.04545454545454546</v>
+      </c>
+      <c r="I25" t="n">
+        <v>4.098621877985489</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0.4090909090909091</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>24</v>
+      </c>
+      <c r="C26" t="n">
+        <v>5</v>
+      </c>
+      <c r="D26" t="n">
+        <v>9</v>
+      </c>
+      <c r="E26" t="n">
+        <v>9</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="I26" t="n">
+        <v>4.08048554939735</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0.2083333333333333</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>19</v>
+      </c>
+      <c r="C27" t="n">
+        <v>5</v>
+      </c>
+      <c r="D27" t="n">
+        <v>5</v>
+      </c>
+      <c r="E27" t="n">
+        <v>7</v>
+      </c>
+      <c r="F27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0.1578947368421053</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0.2631578947368421</v>
+      </c>
+      <c r="I27" t="n">
+        <v>4.356886060060658</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0.2631578947368421</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>25</v>
+      </c>
+      <c r="C28" t="n">
+        <v>8</v>
+      </c>
+      <c r="D28" t="n">
+        <v>8</v>
+      </c>
+      <c r="E28" t="n">
+        <v>7</v>
+      </c>
+      <c r="F28" t="n">
+        <v>2</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="I28" t="n">
+        <v>4.725815626252608</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Morocco</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>22</v>
+      </c>
+      <c r="C29" t="n">
+        <v>4</v>
+      </c>
+      <c r="D29" t="n">
+        <v>9</v>
+      </c>
+      <c r="E29" t="n">
+        <v>8</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0.2727272727272727</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0.1363636363636364</v>
+      </c>
+      <c r="I29" t="n">
+        <v>4.541296799745269</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0.1818181818181818</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>22</v>
+      </c>
+      <c r="C30" t="n">
+        <v>7</v>
+      </c>
+      <c r="D30" t="n">
+        <v>8</v>
+      </c>
+      <c r="E30" t="n">
+        <v>6</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0.04545454545454546</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0.1818181818181818</v>
+      </c>
+      <c r="I30" t="n">
+        <v>3.826315805143722</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0.3181818181818182</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>17</v>
+      </c>
+      <c r="C31" t="n">
+        <v>2</v>
+      </c>
+      <c r="D31" t="n">
+        <v>7</v>
+      </c>
+      <c r="E31" t="n">
+        <v>7</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0.1176470588235294</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="I31" t="n">
+        <v>4.570525777451971</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0.1176470588235294</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>25</v>
+      </c>
+      <c r="C32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D32" t="n">
+        <v>11</v>
+      </c>
+      <c r="E32" t="n">
+        <v>9</v>
+      </c>
+      <c r="F32" t="n">
+        <v>2</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="I32" t="n">
+        <v>3.056686659331199</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>20</v>
+      </c>
+      <c r="C33" t="n">
+        <v>4</v>
+      </c>
+      <c r="D33" t="n">
+        <v>6</v>
+      </c>
+      <c r="E33" t="n">
+        <v>9</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I33" t="n">
+        <v>3.837488213594106</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>23</v>
+      </c>
+      <c r="C34" t="n">
+        <v>5</v>
+      </c>
+      <c r="D34" t="n">
+        <v>9</v>
+      </c>
+      <c r="E34" t="n">
+        <v>7</v>
+      </c>
+      <c r="F34" t="n">
+        <v>2</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0.08695652173913043</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0.3043478260869565</v>
+      </c>
+      <c r="I34" t="n">
+        <v>4.809411064008636</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0.2173913043478261</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>22</v>
+      </c>
+      <c r="C35" t="n">
+        <v>7</v>
+      </c>
+      <c r="D35" t="n">
+        <v>6</v>
+      </c>
+      <c r="E35" t="n">
+        <v>7</v>
+      </c>
+      <c r="F35" t="n">
+        <v>2</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0.09090909090909091</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0.1818181818181818</v>
+      </c>
+      <c r="I35" t="n">
+        <v>4.480114794447635</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0.3181818181818182</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>21</v>
+      </c>
+      <c r="C36" t="n">
+        <v>6</v>
+      </c>
+      <c r="D36" t="n">
+        <v>4</v>
+      </c>
+      <c r="E36" t="n">
+        <v>9</v>
+      </c>
+      <c r="F36" t="n">
+        <v>2</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0.09523809523809523</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="I36" t="n">
+        <v>4.652700188881617</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0.2857142857142857</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Saudi Arabia</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>15</v>
+      </c>
+      <c r="C37" t="n">
+        <v>5</v>
+      </c>
+      <c r="D37" t="n">
+        <v>3</v>
+      </c>
+      <c r="E37" t="n">
+        <v>6</v>
+      </c>
+      <c r="F37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0.06666666666666667</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0.1333333333333333</v>
+      </c>
+      <c r="I37" t="n">
+        <v>3.60951124510943</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Scotland</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>22</v>
+      </c>
+      <c r="C38" t="n">
+        <v>6</v>
+      </c>
+      <c r="D38" t="n">
+        <v>5</v>
+      </c>
+      <c r="E38" t="n">
+        <v>9</v>
+      </c>
+      <c r="F38" t="n">
+        <v>2</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0.09090909090909091</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0.1818181818181818</v>
+      </c>
+      <c r="I38" t="n">
+        <v>4.853034932075809</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0.2727272727272727</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>21</v>
+      </c>
+      <c r="C39" t="n">
+        <v>7</v>
+      </c>
+      <c r="D39" t="n">
+        <v>4</v>
+      </c>
+      <c r="E39" t="n">
+        <v>7</v>
+      </c>
+      <c r="F39" t="n">
+        <v>3</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="I39" t="n">
+        <v>5.04880938345628</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>19</v>
+      </c>
+      <c r="C40" t="n">
+        <v>8</v>
+      </c>
+      <c r="D40" t="n">
+        <v>5</v>
+      </c>
+      <c r="E40" t="n">
+        <v>5</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0.2105263157894737</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0.1052631578947368</v>
+      </c>
+      <c r="I40" t="n">
+        <v>4.399627841783761</v>
+      </c>
+      <c r="J40" t="n">
+        <v>0.4210526315789473</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>20</v>
+      </c>
+      <c r="C41" t="n">
+        <v>3</v>
+      </c>
+      <c r="D41" t="n">
+        <v>9</v>
+      </c>
+      <c r="E41" t="n">
+        <v>7</v>
+      </c>
+      <c r="F41" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="I41" t="n">
+        <v>3.688888008172937</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>24</v>
+      </c>
+      <c r="C42" t="n">
+        <v>8</v>
+      </c>
+      <c r="D42" t="n">
+        <v>7</v>
+      </c>
+      <c r="E42" t="n">
+        <v>7</v>
+      </c>
+      <c r="F42" t="n">
+        <v>2</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0.2083333333333333</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0.08333333333333333</v>
+      </c>
+      <c r="I42" t="n">
+        <v>4.014240953752354</v>
+      </c>
+      <c r="J42" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>21</v>
+      </c>
+      <c r="C43" t="n">
+        <v>4</v>
+      </c>
+      <c r="D43" t="n">
+        <v>7</v>
+      </c>
+      <c r="E43" t="n">
+        <v>8</v>
+      </c>
+      <c r="F43" t="n">
+        <v>2</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0.09523809523809523</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0.09523809523809523</v>
+      </c>
+      <c r="I43" t="n">
+        <v>3.785309951453305</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0.1904761904761905</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>23</v>
+      </c>
+      <c r="C44" t="n">
+        <v>7</v>
+      </c>
+      <c r="D44" t="n">
+        <v>8</v>
+      </c>
+      <c r="E44" t="n">
+        <v>7</v>
+      </c>
+      <c r="F44" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0.04347826086956522</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0.2173913043478261</v>
+      </c>
+      <c r="I44" t="n">
+        <v>3.629588550163539</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0.3043478260869565</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Tunisia</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>21</v>
+      </c>
+      <c r="C45" t="n">
+        <v>4</v>
+      </c>
+      <c r="D45" t="n">
+        <v>8</v>
+      </c>
+      <c r="E45" t="n">
+        <v>7</v>
+      </c>
+      <c r="F45" t="n">
+        <v>2</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0.09523809523809523</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0.09523809523809523</v>
+      </c>
+      <c r="I45" t="n">
+        <v>3.404478842712375</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0.1904761904761905</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Turkiye</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>23</v>
+      </c>
+      <c r="C46" t="n">
+        <v>9</v>
+      </c>
+      <c r="D46" t="n">
+        <v>5</v>
+      </c>
+      <c r="E46" t="n">
+        <v>8</v>
+      </c>
+      <c r="F46" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0.1739130434782609</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0.04347826086956522</v>
+      </c>
+      <c r="I46" t="n">
+        <v>3.44866360093458</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0.391304347826087</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>24</v>
+      </c>
+      <c r="C47" t="n">
+        <v>7</v>
+      </c>
+      <c r="D47" t="n">
+        <v>5</v>
+      </c>
+      <c r="E47" t="n">
+        <v>10</v>
+      </c>
+      <c r="F47" t="n">
+        <v>2</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0.04166666666666666</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0.04166666666666666</v>
+      </c>
+      <c r="I47" t="n">
+        <v>3.33514443552256</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0.2916666666666667</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Uruguay</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>18</v>
+      </c>
+      <c r="C48" t="n">
+        <v>4</v>
+      </c>
+      <c r="D48" t="n">
+        <v>7</v>
+      </c>
+      <c r="E48" t="n">
+        <v>5</v>
+      </c>
+      <c r="F48" t="n">
+        <v>2</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="I48" t="n">
+        <v>3.547990317647111</v>
+      </c>
+      <c r="J48" t="n">
+        <v>0.2222222222222222</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Uzbekistan</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>19</v>
+      </c>
+      <c r="C49" t="n">
+        <v>3</v>
+      </c>
+      <c r="D49" t="n">
+        <v>8</v>
+      </c>
+      <c r="E49" t="n">
+        <v>6</v>
+      </c>
+      <c r="F49" t="n">
+        <v>2</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0.2105263157894737</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0.1578947368421053</v>
+      </c>
+      <c r="I49" t="n">
+        <v>4.546060565661952</v>
+      </c>
+      <c r="J49" t="n">
+        <v>0.1578947368421053</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>